<commit_message>
Update QnA Excel output
</commit_message>
<xml_diff>
--- a/output/QnA.xlsx
+++ b/output/QnA.xlsx
@@ -460,24 +460,24 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>What disciplines does Indian Knowledge Systems (IKS) encompass according to the text?</t>
+          <t>What disciplines does Indian Knowledge Systems (IKS) encompass?</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Science, philosophy, medicine, mathematics, arts, and environmental management.</t>
+          <t>science, philosophy, medicine, mathematics, arts, and environmental management</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>How does the text describe the relevance of IKS in the 21st century?</t>
+          <t>How does IKS approach knowledge integration?</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>They provide holistic solutions for health, environment, society, and personal well-being, offering integrated, sustainable knowledge that addresses both material progress and spiritual well-being.</t>
+          <t>inherently holistic, integrating various streams of knowledge to promote harmony between human life, society, and nature</t>
         </is>
       </c>
     </row>
@@ -538,24 +538,24 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>पाठ के अनुसार भारतीय ज्ञान प्रणालियों (आईकेएस) में कौन सी अनुशासन शामिल हैं?</t>
+          <t>भारतीय ज्ञान प्रणालियों (आईकेएस) में कौन सी अनुशासन शामिल हैं?</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>विज्ञान, दर्शन, चिकित्सा, गणित, कला, और पर्यावरण प्रबंधन।</t>
+          <t>विज्ञान, दर्शन, चिकित्सा, गणित, कला, और पर्यावरण प्रबंधन</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>पाठ 21 वीं शताब्दी में आईकेएस की प्रासंगिकता का वर्णन कैसे करता है?</t>
+          <t>आईसीएस ज्ञान एकीकरण के लिए कैसे दृष्टिकोण करता है?</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>वे स्वास्थ्य, पर्यावरण, समाज और व्यक्तिगत कल्याण के लिए समग्र समाधान प्रदान करते हैं, एकीकृत, सतत ज्ञान प्रदान करते हैं जो भौतिक प्रगति और आध्यात्मिक कल्याण दोनों को संबोधित करता है।</t>
+          <t>अंतर्निहित रूप से समग्र, मानव जीवन, समाज और प्रकृति के बीच सामंजस्य को बढ़ावा देने के लिए ज्ञान के विभिन्न प्रवाहों को एकीकृत</t>
         </is>
       </c>
     </row>
@@ -616,24 +616,24 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>भारतीय ज्ञान प्रणाली (आईकेएस) या संदर्भानुसार कोणते संदर्भ घेतात?</t>
+          <t>भारतीय ज्ञान प्रणाली (आईकेएस) कोणते अनुशासनांना समावेश आहे?</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>विज्ञान, दर्शन, औषध, गणित, कला आणि पर्यावरण प्रबंधन.</t>
+          <t>विज्ञान, दर्शन, औषध, गणित, कला आणि पर्यावरण प्रबंधन</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>21 वी शताब्दीत आईकेएसचे महत्व कसा वर्णन करतो?</t>
+          <t>IKS ज्ञान एकीकरण कसा करतो?</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>हे स्वास्थ्य, पर्यावरण, समाज आणि व्यक्तिगत कल्याणसाठी समग्र समाधान प्रदान करते आणि सामंजस्यपूर्ण, स्थिर ज्ञान प्रदान करते, जो भौतिक प्रगती आणि आध्यात्मिक कल्याण कोणाला लक्ष देतो.</t>
+          <t>मानव जीवन, समाज आणि प्राकृतिक संतुलन प्रोत्साहित करण्यासाठी विविध ज्ञान प्रवाह एकीकृत होय.</t>
         </is>
       </c>
     </row>

</xml_diff>